<commit_message>
Fix rolling 12 brand trends and update Night Vision outputs
</commit_message>
<xml_diff>
--- a/product_dashboard/data/non_code_categories/Night Vision Monoculars/outputs/Night_Vision_Market_Analysis_202603.xlsx
+++ b/product_dashboard/data/non_code_categories/Night Vision Monoculars/outputs/Night_Vision_Market_Analysis_202603.xlsx
@@ -10,6 +10,8 @@
     <sheet name="Price Tiers" sheetId="5" r:id="rId5"/>
     <sheet name="All ASINs" sheetId="6" r:id="rId6"/>
     <sheet name="Metadata" sheetId="7" r:id="rId7"/>
+    <sheet name="Topdon" sheetId="8" r:id="rId8"/>
+    <sheet name="Guide Sensmart" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -57718,7 +57720,7 @@
         <v>Generated At</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-03-29T16:46:43.774Z</v>
+        <v>2026-03-30T21:26:07.949Z</v>
       </c>
     </row>
     <row r="7">
@@ -57734,4 +57736,320 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L3"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="80.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="34.83203125" customWidth="1"/>
+    <col min="11" max="11" width="25.83203125" customWidth="1"/>
+    <col min="12" max="12" width="21.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ASIN</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Title</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Brand</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Price</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Monthly Rev</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Monthly Units</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Avg Rating</v>
+      </c>
+      <c r="I1" t="str">
+        <v># of Reviews</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Link</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Subcategory</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Size Tier</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>B0D56CNCW1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>TOPDON TS004 Thermal Imaging Monocular, 320 x 240 TISR 256 x 192 IR Resolution, Supported Wireless Connection, 13mm 50Hz Thermal Night Vision with 11h Battery Life, IP67 Monocular for Hunting</v>
+      </c>
+      <c r="C2" t="str">
+        <v>TOPDON</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Night Vision Monoculars</v>
+      </c>
+      <c r="E2">
+        <v>409.99</v>
+      </c>
+      <c r="F2">
+        <v>429870.86</v>
+      </c>
+      <c r="G2">
+        <v>1058</v>
+      </c>
+      <c r="H2">
+        <v>4.5</v>
+      </c>
+      <c r="I2">
+        <v>274</v>
+      </c>
+      <c r="J2" t="str">
+        <v>https://amazon.com/dp/B0D56CNCW1</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Night Vision Monoculars</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Large Standard-Size</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>B0FW4H9MXB</v>
+      </c>
+      <c r="B3" t="str">
+        <v>TOPDON TS004 Pro Thermal Imaging Monocular, 512 x 384 TISR 384 x 288 IR Resolution, Supported Wireless Connection, 19mm 50Hz Thermal Night Vision with 11h Battery Life, IP67 Monocular for Hunting</v>
+      </c>
+      <c r="C3" t="str">
+        <v>TOPDON</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Night Vision Monoculars</v>
+      </c>
+      <c r="E3">
+        <v>899</v>
+      </c>
+      <c r="F3">
+        <v>53340.74</v>
+      </c>
+      <c r="G3">
+        <v>61</v>
+      </c>
+      <c r="H3">
+        <v>4.5</v>
+      </c>
+      <c r="I3">
+        <v>274</v>
+      </c>
+      <c r="J3" t="str">
+        <v>https://amazon.com/dp/B0FW4H9MXB</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Night Vision Monoculars</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Large Standard-Size</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L4"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="80.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="34.83203125" customWidth="1"/>
+    <col min="11" max="11" width="25.83203125" customWidth="1"/>
+    <col min="12" max="12" width="21.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ASIN</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Title</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Brand</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Price</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Monthly Rev</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Monthly Units</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Avg Rating</v>
+      </c>
+      <c r="I1" t="str">
+        <v># of Reviews</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Link</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Subcategory</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Size Tier</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>B0FDH7FLVK</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Guide TE211 Thermal Monocular, 10mm Focal Lens, 256×192(50Hz) 12μm Handheld Night Vision Infrared Scope with 6-Hour Battery Life, 20W Quick Charging, Thermal Imaging Monocular for Hunting, Outdoor</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Guide Sensmart</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Night Vision Monoculars</v>
+      </c>
+      <c r="E2">
+        <v>519</v>
+      </c>
+      <c r="F2">
+        <v>1988.44</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="str">
+        <v>https://amazon.com/dp/B0FDH7FLVK</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Night Vision Monoculars</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Large Standard-Size</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>B0C4YK81C2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Guide Sensmart TK421 Thermal Imaging Monocular for Night Hunting -400x300 (50 Hz) High Sensitivity Thermal Vision Monocular, 6.8X Digtal Zoom &amp; 1800yd Search Range</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Guide Sensmart</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Night Vision Monoculars</v>
+      </c>
+      <c r="E3">
+        <v>949</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3">
+        <v>5</v>
+      </c>
+      <c r="J3" t="str">
+        <v>https://amazon.com/dp/B0C4YK81C2</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Night Vision Monoculars</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Large Standard-Size</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>B0B1MYC1PL</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Guide Sensmart TK431 Thermal Vision Monocular – Night Vision for Hunting, 2.3X Optical Zoom, 9.2X Digital Zoom, 400x300 Resolution, 1550yd Detection Range, WiFi Video Streaming, Waterproof</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Guide Sensmart</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Night Vision Monoculars</v>
+      </c>
+      <c r="E4">
+        <v>999</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>5</v>
+      </c>
+      <c r="I4">
+        <v>5</v>
+      </c>
+      <c r="J4" t="str">
+        <v>https://amazon.com/dp/B0B1MYC1PL</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Night Vision Monoculars</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Large Standard-Size</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>